<commit_message>
Se agregan comentarios importantes
</commit_message>
<xml_diff>
--- a/mia07_t3_tra_resultados_viterbi.xlsx
+++ b/mia07_t3_tra_resultados_viterbi.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NCMS000</t>
+          <t>AQ0MS0</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -474,7 +474,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2.827818374535177e-08</v>
+        <v>1.295582484193506e-09</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -492,7 +492,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NCMP000</t>
+          <t>Fp</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -514,16 +514,16 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>4.107075865754602e-15</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>3.529518322132861e-16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fp</t>
+          <t>DA0MS0</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -533,7 +533,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>2.779888150251198e-06</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -548,20 +548,20 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>3.529518322132861e-16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SPS00</t>
+          <t>NCFS000</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>1.988063133517315e-05</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -573,7 +573,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>5.440257583147429e-12</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -585,14 +585,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NCFS000</t>
+          <t>SPS00</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1.988063133517315e-05</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -604,7 +604,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>5.440257583147429e-12</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -616,11 +616,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AQ0CS0</t>
+          <t>VMIP3S0</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>0.0012941074971961</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -632,7 +632,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>6.385259012197449e-11</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DA0MS0</t>
+          <t>NCMP000</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -657,7 +657,7 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>2.779888150251198e-06</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -669,7 +669,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>4.107075865754602e-15</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -678,11 +678,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>VMIP3S0</t>
+          <t>AQ0CS0</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0012941074971961</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -694,7 +694,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>6.385259012197449e-11</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -709,7 +709,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AQ0MS0</t>
+          <t>NCMS000</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -722,7 +722,7 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1.295582484193506e-09</v>
+        <v>2.827818374535177e-08</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>

</xml_diff>